<commit_message>
Selected Work: bump citations_asof to August 2026
The last Scholar hand-refresh was July; the page's date footnote had
drifted a month stale. No count changes, just the as-of date on the
Meta sheet.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/selected-work/data/publications.xlsx
+++ b/selected-work/data/publications.xlsx
@@ -1,23 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Publications" sheetId="1" r:id="rId1"/>
-    <sheet name="Areas" sheetId="2" r:id="rId2"/>
-    <sheet name="Reports" sheetId="3" r:id="rId3"/>
-    <sheet name="Meta" sheetId="4" r:id="rId4"/>
+    <sheet name="Publications" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Areas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Reports" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Meta" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+  <si>
+    <t xml:space="preserve">August 2026</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -27,12 +35,12 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <b/>
     </font>
   </fonts>
   <fills count="2">
@@ -353,11 +361,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K37"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>id</t>
@@ -420,7 +428,7 @@
           <t>BOOK2025</t>
         </is>
       </c>
-      <c r="B2">
+      <c r="B2" t="n">
         <v>2025</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -468,7 +476,7 @@
           <t>AGEPRIS2023</t>
         </is>
       </c>
-      <c r="B3">
+      <c r="B3" t="n">
         <v>2023</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -511,7 +519,7 @@
           <t>ANNREV2021</t>
         </is>
       </c>
-      <c r="B4">
+      <c r="B4" t="n">
         <v>2021</v>
       </c>
       <c r="C4" t="inlineStr">
@@ -552,7 +560,7 @@
       <c r="J4" t="b">
         <v>1</v>
       </c>
-      <c r="K4">
+      <c r="K4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -562,7 +570,7 @@
           <t>ENDLIFE2021</t>
         </is>
       </c>
-      <c r="B5">
+      <c r="B5" t="n">
         <v>2021</v>
       </c>
       <c r="C5" t="inlineStr">
@@ -610,7 +618,7 @@
           <t>CONFID2018</t>
         </is>
       </c>
-      <c r="B6">
+      <c r="B6" t="n">
         <v>2018</v>
       </c>
       <c r="C6" t="inlineStr">
@@ -658,7 +666,7 @@
           <t>COMPREL2018</t>
         </is>
       </c>
-      <c r="B7">
+      <c r="B7" t="n">
         <v>2018</v>
       </c>
       <c r="C7" t="inlineStr">
@@ -699,7 +707,7 @@
       <c r="J7" t="b">
         <v>1</v>
       </c>
-      <c r="K7">
+      <c r="K7" t="n">
         <v>2</v>
       </c>
     </row>
@@ -709,7 +717,7 @@
           <t>PATRON2015</t>
         </is>
       </c>
-      <c r="B8">
+      <c r="B8" t="n">
         <v>2015</v>
       </c>
       <c r="C8" t="inlineStr">
@@ -757,7 +765,7 @@
           <t>ORB2015</t>
         </is>
       </c>
-      <c r="B9">
+      <c r="B9" t="n">
         <v>2015</v>
       </c>
       <c r="C9" t="inlineStr">
@@ -805,7 +813,7 @@
           <t>ELDERS2015</t>
         </is>
       </c>
-      <c r="B10">
+      <c r="B10" t="n">
         <v>2015</v>
       </c>
       <c r="C10" t="inlineStr">
@@ -848,7 +856,7 @@
           <t>MISINFO2014</t>
         </is>
       </c>
-      <c r="B11">
+      <c r="B11" t="n">
         <v>2014</v>
       </c>
       <c r="C11" t="inlineStr">
@@ -891,7 +899,7 @@
           <t>CAREGIV2014</t>
         </is>
       </c>
-      <c r="B12">
+      <c r="B12" t="n">
         <v>2014</v>
       </c>
       <c r="C12" t="inlineStr">
@@ -939,7 +947,7 @@
           <t>ELDMAL2012</t>
         </is>
       </c>
-      <c r="B13">
+      <c r="B13" t="n">
         <v>2012</v>
       </c>
       <c r="C13" t="inlineStr">
@@ -987,7 +995,7 @@
           <t>EMYOUTH2023</t>
         </is>
       </c>
-      <c r="B14">
+      <c r="B14" t="n">
         <v>2023</v>
       </c>
       <c r="C14" t="inlineStr">
@@ -1028,7 +1036,7 @@
       <c r="J14" t="b">
         <v>1</v>
       </c>
-      <c r="K14">
+      <c r="K14" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1038,7 +1046,7 @@
           <t>EMERGING2022</t>
         </is>
       </c>
-      <c r="B15">
+      <c r="B15" t="n">
         <v>2022</v>
       </c>
       <c r="C15" t="inlineStr">
@@ -1079,7 +1087,7 @@
       <c r="J15" t="b">
         <v>1</v>
       </c>
-      <c r="K15">
+      <c r="K15" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1089,7 +1097,7 @@
           <t>DEADLY2022</t>
         </is>
       </c>
-      <c r="B16">
+      <c r="B16" t="n">
         <v>2022</v>
       </c>
       <c r="C16" t="inlineStr">
@@ -1137,7 +1145,7 @@
           <t>VICTIM2021</t>
         </is>
       </c>
-      <c r="B17">
+      <c r="B17" t="n">
         <v>2021</v>
       </c>
       <c r="C17" t="inlineStr">
@@ -1185,7 +1193,7 @@
           <t>SURGERY2021</t>
         </is>
       </c>
-      <c r="B18">
+      <c r="B18" t="n">
         <v>2021</v>
       </c>
       <c r="C18" t="inlineStr">
@@ -1233,7 +1241,7 @@
           <t>DRUGTEST2021</t>
         </is>
       </c>
-      <c r="B19">
+      <c r="B19" t="n">
         <v>2021</v>
       </c>
       <c r="C19" t="inlineStr">
@@ -1281,7 +1289,7 @@
           <t>RNR2019</t>
         </is>
       </c>
-      <c r="B20">
+      <c r="B20" t="n">
         <v>2019</v>
       </c>
       <c r="C20" t="inlineStr">
@@ -1322,7 +1330,7 @@
       <c r="J20" t="b">
         <v>1</v>
       </c>
-      <c r="K20">
+      <c r="K20" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1332,7 +1340,7 @@
           <t>VICTREC2018</t>
         </is>
       </c>
-      <c r="B21">
+      <c r="B21" t="n">
         <v>2018</v>
       </c>
       <c r="C21" t="inlineStr">
@@ -1373,7 +1381,7 @@
       <c r="J21" t="b">
         <v>1</v>
       </c>
-      <c r="K21">
+      <c r="K21" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1383,7 +1391,7 @@
           <t>ABSENT2018</t>
         </is>
       </c>
-      <c r="B22">
+      <c r="B22" t="n">
         <v>2018</v>
       </c>
       <c r="C22" t="inlineStr">
@@ -1431,7 +1439,7 @@
           <t>CPV2018</t>
         </is>
       </c>
-      <c r="B23">
+      <c r="B23" t="n">
         <v>2018</v>
       </c>
       <c r="C23" t="inlineStr">
@@ -1479,7 +1487,7 @@
           <t>CPVCHAP2018</t>
         </is>
       </c>
-      <c r="B24">
+      <c r="B24" t="n">
         <v>2018</v>
       </c>
       <c r="C24" t="inlineStr">
@@ -1522,7 +1530,7 @@
           <t>MAILSURV2015</t>
         </is>
       </c>
-      <c r="B25">
+      <c r="B25" t="n">
         <v>2015</v>
       </c>
       <c r="C25" t="inlineStr">
@@ -1565,7 +1573,7 @@
           <t>WEAPONS2010</t>
         </is>
       </c>
-      <c r="B26">
+      <c r="B26" t="n">
         <v>2010</v>
       </c>
       <c r="C26" t="inlineStr">
@@ -1613,7 +1621,7 @@
           <t>STORY2025</t>
         </is>
       </c>
-      <c r="B27">
+      <c r="B27" t="n">
         <v>2025</v>
       </c>
       <c r="C27" t="inlineStr">
@@ -1654,7 +1662,7 @@
       <c r="J27" t="b">
         <v>1</v>
       </c>
-      <c r="K27">
+      <c r="K27" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1664,7 +1672,7 @@
           <t>LHB402018</t>
         </is>
       </c>
-      <c r="B28">
+      <c r="B28" t="n">
         <v>2018</v>
       </c>
       <c r="C28" t="inlineStr">
@@ -1705,7 +1713,7 @@
       <c r="J28" t="b">
         <v>1</v>
       </c>
-      <c r="K28">
+      <c r="K28" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1715,7 +1723,7 @@
           <t>OBESITY2017</t>
         </is>
       </c>
-      <c r="B29">
+      <c r="B29" t="n">
         <v>2017</v>
       </c>
       <c r="C29" t="inlineStr">
@@ -1763,7 +1771,7 @@
           <t>DISCUSS2013</t>
         </is>
       </c>
-      <c r="B30">
+      <c r="B30" t="n">
         <v>2013</v>
       </c>
       <c r="C30" t="inlineStr">
@@ -1811,7 +1819,7 @@
           <t>EPICRIM2022</t>
         </is>
       </c>
-      <c r="B31">
+      <c r="B31" t="n">
         <v>2022</v>
       </c>
       <c r="C31" t="inlineStr">
@@ -1859,7 +1867,7 @@
           <t>LAWWELL2016</t>
         </is>
       </c>
-      <c r="B32">
+      <c r="B32" t="n">
         <v>2016</v>
       </c>
       <c r="C32" t="inlineStr">
@@ -1907,7 +1915,7 @@
           <t>DUKE2015</t>
         </is>
       </c>
-      <c r="B33">
+      <c r="B33" t="n">
         <v>2015</v>
       </c>
       <c r="C33" t="inlineStr">
@@ -1948,7 +1956,7 @@
       <c r="J33" t="b">
         <v>1</v>
       </c>
-      <c r="K33">
+      <c r="K33" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1958,7 +1966,7 @@
           <t>PARAPH2014</t>
         </is>
       </c>
-      <c r="B34">
+      <c r="B34" t="n">
         <v>2014</v>
       </c>
       <c r="C34" t="inlineStr">
@@ -2006,7 +2014,7 @@
           <t>VOICEID2013</t>
         </is>
       </c>
-      <c r="B35">
+      <c r="B35" t="n">
         <v>2013</v>
       </c>
       <c r="C35" t="inlineStr">
@@ -2054,7 +2062,7 @@
           <t>WHISTLE2011</t>
         </is>
       </c>
-      <c r="B36">
+      <c r="B36" t="n">
         <v>2011</v>
       </c>
       <c r="C36" t="inlineStr">
@@ -2097,7 +2105,7 @@
           <t>JELS2009</t>
         </is>
       </c>
-      <c r="B37">
+      <c r="B37" t="n">
         <v>2009</v>
       </c>
       <c r="C37" t="inlineStr">
@@ -2138,21 +2146,22 @@
       <c r="J37" t="b">
         <v>1</v>
       </c>
-      <c r="K37">
+      <c r="K37" t="n">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>key</t>
@@ -2210,7 +2219,7 @@
           <t>How the legal system meets older adults: as litigants, victims, caregivers, and prisoners.</t>
         </is>
       </c>
-      <c r="F2">
+      <c r="F2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2240,7 +2249,7 @@
           <t>Diversion, risk and needs, and the program features that change outcomes for young people in the system.</t>
         </is>
       </c>
-      <c r="F3">
+      <c r="F3" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2270,7 +2279,7 @@
           <t>Helping courts measure, understand, and communicate the story of their own work.</t>
         </is>
       </c>
-      <c r="F4">
+      <c r="F4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2300,21 +2309,22 @@
           <t>Empirical answers to legal questions, from arbitration outcomes to voice identification evidence.</t>
         </is>
       </c>
-      <c r="F5">
+      <c r="F5" t="n">
         <v>4</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D22"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>org</t>
@@ -2695,15 +2705,16 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>key</t>
@@ -2733,10 +2744,8 @@
           <t>citations_asof</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>July 2026</t>
-        </is>
+      <c r="B3" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -2801,5 +2810,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>